<commit_message>
chore: update dropdowns workbook and refine module2 rows
</commit_message>
<xml_diff>
--- a/public/dropdowns.xlsx
+++ b/public/dropdowns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tudor\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C117207B-E6BA-43EB-B1A2-B5CE195A7845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E98319-035B-49F5-9D85-3E4FC1AD4A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="830" firstSheet="11" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Construction Type" sheetId="8" r:id="rId1"/>
@@ -27,14 +27,23 @@
     <sheet name="Group E" sheetId="19" r:id="rId12"/>
     <sheet name="Group F-1" sheetId="20" r:id="rId13"/>
     <sheet name="Group F-2" sheetId="21" r:id="rId14"/>
-    <sheet name="Group M" sheetId="22" r:id="rId15"/>
-    <sheet name="Group R-1" sheetId="23" r:id="rId16"/>
-    <sheet name="Group R-2" sheetId="24" r:id="rId17"/>
-    <sheet name="Group R-3" sheetId="25" r:id="rId18"/>
-    <sheet name="Group R-4" sheetId="26" r:id="rId19"/>
-    <sheet name="Group S-1" sheetId="27" r:id="rId20"/>
-    <sheet name="Group S-2" sheetId="28" r:id="rId21"/>
-    <sheet name="Group U" sheetId="29" r:id="rId22"/>
+    <sheet name="Group H-1" sheetId="34" r:id="rId15"/>
+    <sheet name="Group H-2" sheetId="33" r:id="rId16"/>
+    <sheet name="Group H-3" sheetId="31" r:id="rId17"/>
+    <sheet name="Group H-4" sheetId="32" r:id="rId18"/>
+    <sheet name="Group H-5" sheetId="30" r:id="rId19"/>
+    <sheet name="Group I-1" sheetId="35" r:id="rId20"/>
+    <sheet name="Group I-2" sheetId="36" r:id="rId21"/>
+    <sheet name="Group I-3" sheetId="37" r:id="rId22"/>
+    <sheet name="Group I-4" sheetId="38" r:id="rId23"/>
+    <sheet name="Group M" sheetId="22" r:id="rId24"/>
+    <sheet name="Group R-1" sheetId="23" r:id="rId25"/>
+    <sheet name="Group R-2" sheetId="24" r:id="rId26"/>
+    <sheet name="Group R-3" sheetId="25" r:id="rId27"/>
+    <sheet name="Group R-4" sheetId="26" r:id="rId28"/>
+    <sheet name="Group S-1" sheetId="27" r:id="rId29"/>
+    <sheet name="Group S-2" sheetId="28" r:id="rId30"/>
+    <sheet name="Group U" sheetId="29" r:id="rId31"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="350">
   <si>
     <t>Occupancy</t>
   </si>
@@ -931,6 +940,177 @@
   </si>
   <si>
     <t>Woodworking (cabinet)</t>
+  </si>
+  <si>
+    <t>Group H-1</t>
+  </si>
+  <si>
+    <t>Group H-2</t>
+  </si>
+  <si>
+    <t>Group H-3</t>
+  </si>
+  <si>
+    <t>Group H-4</t>
+  </si>
+  <si>
+    <t>Group H-5</t>
+  </si>
+  <si>
+    <t>Group I-1</t>
+  </si>
+  <si>
+    <t>Group I-2</t>
+  </si>
+  <si>
+    <t>Group I-3</t>
+  </si>
+  <si>
+    <t>Group I-4</t>
+  </si>
+  <si>
+    <t>Detonable pyrophoric materials</t>
+  </si>
+  <si>
+    <t>Division 1.1 Explosives</t>
+  </si>
+  <si>
+    <t>Division 1.2 Explosives</t>
+  </si>
+  <si>
+    <t>Division 1.3 Explosives</t>
+  </si>
+  <si>
+    <t>Division 1.4 Explosives</t>
+  </si>
+  <si>
+    <t>Division 1.5 Explosives</t>
+  </si>
+  <si>
+    <t>Division 1.6 Explosives</t>
+  </si>
+  <si>
+    <t>Organic peroxides, unclassified detonable</t>
+  </si>
+  <si>
+    <t>Oxidizers, Class 4</t>
+  </si>
+  <si>
+    <t>Unstable (reactive) materials, Class 3 detonable and Class 4</t>
+  </si>
+  <si>
+    <t>Class I, II or IIIA flammable or combustible liquids</t>
+  </si>
+  <si>
+    <t>Cryogenic fluids, flammable</t>
+  </si>
+  <si>
+    <t>Category 1A flammable gases</t>
+  </si>
+  <si>
+    <t>Category 1B flammable gases (BV &gt;3.9 inches per second)</t>
+  </si>
+  <si>
+    <t>Organic peroxides, Class I</t>
+  </si>
+  <si>
+    <t>Oxidizers, Class 3 in open containers or systems (&gt;15 lbs/psi)</t>
+  </si>
+  <si>
+    <t>Pyrophoric liquids, solids and gases, nondetonable</t>
+  </si>
+  <si>
+    <t>Unstable (reactive) materials, Class 3, nondetonable</t>
+  </si>
+  <si>
+    <t>Water-reactive materials, Class 3</t>
+  </si>
+  <si>
+    <t>Combustible dusts (manufactured, generated or used)</t>
+  </si>
+  <si>
+    <t>Consumer fireworks, 1.4G (Class C, Common)</t>
+  </si>
+  <si>
+    <t>Cryogenic fluids, oxidizing</t>
+  </si>
+  <si>
+    <t>Category 1B flammable gases (BV &lt;3.9 inches per second)</t>
+  </si>
+  <si>
+    <t>Flammable solids</t>
+  </si>
+  <si>
+    <t>Organic peroxides, Class II and III</t>
+  </si>
+  <si>
+    <t>Oxidizers, Class 2</t>
+  </si>
+  <si>
+    <t>Oxidizers, Class 3 in closed containers or systems (&lt;15 lbs/psi)</t>
+  </si>
+  <si>
+    <t>Oxidizing gases</t>
+  </si>
+  <si>
+    <t>Unstable (reactive) materials, Class 2</t>
+  </si>
+  <si>
+    <t>Water-reactive materials, Class 2</t>
+  </si>
+  <si>
+    <t>Combustible fibers (manufactured, generated or used)</t>
+  </si>
+  <si>
+    <t>Corrosives</t>
+  </si>
+  <si>
+    <t>Highly toxic materials</t>
+  </si>
+  <si>
+    <t>Toxic materials</t>
+  </si>
+  <si>
+    <t>Semiconductor fabrication, research, and development facilities</t>
+  </si>
+  <si>
+    <t>Foster care facilities</t>
+  </si>
+  <si>
+    <t>Detoxification facilities</t>
+  </si>
+  <si>
+    <t>Hospitals</t>
+  </si>
+  <si>
+    <t>Nursing homes</t>
+  </si>
+  <si>
+    <t>Psychiatric hospitals</t>
+  </si>
+  <si>
+    <t>Correctional centers</t>
+  </si>
+  <si>
+    <t>Detention centers</t>
+  </si>
+  <si>
+    <t>Jails</t>
+  </si>
+  <si>
+    <t>Prerelease centers</t>
+  </si>
+  <si>
+    <t>Prisons</t>
+  </si>
+  <si>
+    <t>Reformatories</t>
+  </si>
+  <si>
+    <t>Adult day care</t>
+  </si>
+  <si>
+    <t>Child day care</t>
   </si>
 </sst>
 </file>
@@ -985,17 +1165,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2380,7 +2564,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFFAF39F-26FB-466F-A77E-23DDCF5708FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEABCD5F-C6CA-4D12-BBF2-B51B507DDF6C}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -2391,85 +2575,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>4</v>
+      <c r="A1" s="5" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
+      <c r="A2" s="5" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>55</v>
+      <c r="A3" s="5" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>74</v>
+      <c r="A4" s="5" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>93</v>
+      <c r="A5" s="5" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>108</v>
+      <c r="A6" s="5" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>121</v>
+      <c r="A7" s="5" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>133</v>
+      <c r="A8" s="5" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>13</v>
+      <c r="A9" s="5" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="3"/>
+      <c r="A10" s="5" t="s">
+        <v>310</v>
+      </c>
     </row>
     <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="3"/>
+      <c r="A11" s="5" t="s">
+        <v>311</v>
+      </c>
     </row>
     <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="3"/>
+      <c r="A12" s="4"/>
     </row>
     <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="3"/>
+      <c r="A13" s="4"/>
     </row>
     <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="3"/>
+      <c r="A14" s="4"/>
     </row>
     <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="3"/>
+      <c r="A15" s="4"/>
     </row>
     <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="3"/>
+      <c r="A16" s="4"/>
     </row>
     <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="3"/>
+      <c r="A17" s="4"/>
     </row>
     <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="3"/>
+      <c r="A18" s="4"/>
     </row>
     <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="3"/>
+      <c r="A19" s="4"/>
     </row>
     <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="3"/>
+      <c r="A20" s="4"/>
     </row>
     <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="3"/>
+      <c r="A21" s="4"/>
     </row>
     <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3"/>
@@ -2570,7 +2758,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4176F08F-2BDE-4395-941C-2CE885F3F67D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4245D1BE-1EB0-494A-B820-59BA0C6B2BEE}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -2581,65 +2769,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>24</v>
+      <c r="A1" s="5" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>39</v>
+      <c r="A2" s="5" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>56</v>
+      <c r="A3" s="5" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>75</v>
+      <c r="A4" s="5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>94</v>
+      <c r="A5" s="5" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>109</v>
+      <c r="A6" s="5" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
+      <c r="A7" s="5" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>13</v>
+      <c r="A8" s="5" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="3"/>
+      <c r="A9" s="5" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="3"/>
+      <c r="A10" s="5" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="3"/>
+      <c r="A11" s="5" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="3"/>
+      <c r="A12" s="5"/>
     </row>
     <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="3"/>
+      <c r="A13" s="5"/>
     </row>
     <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="3"/>
+      <c r="A14" s="5"/>
     </row>
     <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="3"/>
+      <c r="A15" s="5"/>
     </row>
     <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3"/>
@@ -2758,7 +2952,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B36BC44F-D336-4F53-9163-B2C75E177C20}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5F05412-7C00-4D6B-930D-9C115C61832F}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -2769,85 +2963,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
+      <c r="A1" s="5" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>40</v>
+      <c r="A2" s="5" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>57</v>
+      <c r="A3" s="5" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>76</v>
+      <c r="A4" s="5" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>95</v>
+      <c r="A5" s="6" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>110</v>
+      <c r="A6" s="6" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>122</v>
+      <c r="A7" s="6" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>134</v>
+      <c r="A8" s="6" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>145</v>
+      <c r="A9" s="6" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
-        <v>153</v>
+      <c r="A10" s="6" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>161</v>
+      <c r="A11" s="5" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
-        <v>170</v>
+      <c r="A12" s="6" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
-        <v>179</v>
+      <c r="A13" s="6" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A14" s="5"/>
     </row>
     <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A15" s="5"/>
     </row>
     <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="3"/>
+      <c r="A16" s="5"/>
     </row>
     <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="3"/>
+      <c r="A17" s="5"/>
     </row>
     <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="3"/>
@@ -2960,7 +3150,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ACD1348-4F81-4688-9F4A-58D34A85EBF6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75ADD3ED-9BF0-4742-9255-AB21A70433AC}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -2971,84 +3161,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>26</v>
+      <c r="A1" s="5" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>41</v>
+      <c r="A2" s="5" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>58</v>
+      <c r="A3" s="6" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>77</v>
+      <c r="A4" s="5" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="A5" s="5"/>
     </row>
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>95</v>
-      </c>
+      <c r="A6" s="4"/>
     </row>
     <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>110</v>
-      </c>
+      <c r="A7" s="4"/>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>122</v>
-      </c>
+      <c r="A8" s="4"/>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>134</v>
-      </c>
+      <c r="A9" s="4"/>
     </row>
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
-        <v>145</v>
-      </c>
+      <c r="A10" s="3"/>
     </row>
     <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>162</v>
-      </c>
+      <c r="A11" s="3"/>
     </row>
     <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
-        <v>171</v>
-      </c>
+      <c r="A12" s="3"/>
     </row>
     <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
-        <v>180</v>
-      </c>
+      <c r="A13" s="3"/>
     </row>
     <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
-        <v>187</v>
-      </c>
+      <c r="A14" s="3"/>
     </row>
     <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="2" t="s">
-        <v>194</v>
-      </c>
+      <c r="A15" s="3"/>
     </row>
     <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A16" s="3"/>
     </row>
     <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="3"/>
@@ -3164,7 +3330,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9C59B1E-EB67-4C23-8979-195C7EEADBF5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8E39A71-33F8-49A5-BE95-A6815E3F436D}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -3175,49 +3341,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>27</v>
+      <c r="A1" s="5" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>42</v>
+      <c r="A2" s="5" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="A3" s="5"/>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="A4" s="5"/>
     </row>
     <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="A5" s="5"/>
     </row>
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>111</v>
-      </c>
+      <c r="A6" s="5"/>
     </row>
     <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>123</v>
-      </c>
+      <c r="A7" s="3"/>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>135</v>
-      </c>
+      <c r="A8" s="3"/>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="3"/>
     </row>
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3"/>
@@ -3229,10 +3381,10 @@
       <c r="A12" s="3"/>
     </row>
     <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2"/>
+      <c r="A13" s="3"/>
     </row>
     <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2"/>
+      <c r="A14" s="3"/>
     </row>
     <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3"/>
@@ -3398,10 +3550,10 @@
       <c r="A7" s="3"/>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="4"/>
+      <c r="A8" s="3"/>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4"/>
+      <c r="A9" s="3"/>
     </row>
     <row r="27" ht="12.3" x14ac:dyDescent="0.4"/>
     <row r="28" ht="12.3" x14ac:dyDescent="0.4"/>
@@ -3435,244 +3587,63 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C11D53-C013-4501-A6B7-B34906229FB4}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:A52"/>
-  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C121FB28-C97B-4E40-ABF1-EC22E15BB59B}">
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A5" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A6" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A7" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A8" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A9" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="2" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="2" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="2" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A27" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A28" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A29" s="2" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A30" s="2" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A31" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A32" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A33" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A34" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A35" s="2" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A36" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A37" s="2" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A38" s="2" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A39" s="3"/>
-    </row>
-    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A40" s="3"/>
-    </row>
-    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A41" s="3"/>
-    </row>
-    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A42" s="3"/>
-    </row>
-    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A44" s="3"/>
-    </row>
-    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A45" s="3"/>
-    </row>
-    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A46" s="3"/>
-    </row>
-    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A47" s="3"/>
-    </row>
-    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A50" s="3"/>
-    </row>
-    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A51" s="3"/>
-    </row>
-    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A52" s="3"/>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A12" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3680,236 +3651,59 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{968165A6-7FAC-4692-BC4F-B6EE8870C933}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:A52"/>
-  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{968F0942-566C-44A6-9195-32880AC6094B}">
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A5" s="5" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A6" s="5" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="2" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="2" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A27" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A28" s="2" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A29" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A30" s="2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A31" s="2" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A32" s="2" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A33" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A34" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A35" s="3"/>
-    </row>
-    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A36" s="3"/>
-    </row>
-    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A37" s="3"/>
-    </row>
-    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A38" s="3"/>
-    </row>
-    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A39" s="3"/>
-    </row>
-    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A40" s="3"/>
-    </row>
-    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A41" s="3"/>
-    </row>
-    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A42" s="3"/>
-    </row>
-    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A44" s="3"/>
-    </row>
-    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A45" s="3"/>
-    </row>
-    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A46" s="3"/>
-    </row>
-    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A47" s="3"/>
-    </row>
-    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A50" s="3"/>
-    </row>
-    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A51" s="3"/>
-    </row>
-    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
-      <c r="A52" s="3"/>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A12" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3917,7 +3711,114 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C349F70-1ADD-4EC8-9C21-A8161FE0FF5D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBFAD4CF-47B2-447B-B120-C60F80FEE94A}">
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A6" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A7" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A8" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A11" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF3997FA-B9EC-4756-A081-07A605B3469D}">
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A10" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFFAF39F-26FB-466F-A77E-23DDCF5708FD}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -3929,77 +3830,455 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
-        <v>148</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="3"/>
+    </row>
+    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="3"/>
+    </row>
+    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="3"/>
+    </row>
+    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4176F08F-2BDE-4395-941C-2CE885F3F67D}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:A52"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="12.609375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="3"/>
+    </row>
+    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="3"/>
+    </row>
+    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="3"/>
+    </row>
+    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B36BC44F-D336-4F53-9163-B2C75E177C20}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:A52"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="12.609375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
-        <v>190</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
-        <v>197</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -4070,6 +4349,645 @@
     </row>
     <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
       <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ACD1348-4F81-4688-9F4A-58D34A85EBF6}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:A52"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="12.609375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="3"/>
+    </row>
+    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="3"/>
+    </row>
+    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9C59B1E-EB67-4C23-8979-195C7EEADBF5}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:A52"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="12.609375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2"/>
+    </row>
+    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="2"/>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="3"/>
+    </row>
+    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="3"/>
+    </row>
+    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C11D53-C013-4501-A6B7-B34906229FB4}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:A52"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="2" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="2" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
       <c r="A39" s="3"/>
@@ -4214,6 +5132,445 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{968165A6-7FAC-4692-BC4F-B6EE8870C933}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:A52"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C349F70-1ADD-4EC8-9C21-A8161FE0FF5D}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:A52"/>
+  <sheetFormatPr defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="12.609375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="3"/>
+    </row>
+    <row r="28" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="3"/>
+    </row>
+    <row r="35" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="3"/>
+    </row>
+    <row r="40" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A50" s="3"/>
+    </row>
+    <row r="51" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62FBC85-40ED-4BF1-A0EF-AB7D3E2D750F}">
   <sheetPr>
@@ -4232,116 +5589,154 @@
       <c r="B1" s="3"/>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="3"/>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3"/>
     </row>
     <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="3"/>
     </row>
     <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="3"/>
     </row>
     <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="3"/>
     </row>
     <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="B15" s="3"/>
+    </row>
+    <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="B18" s="3"/>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="B19" s="3"/>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
+      <c r="B20" s="3"/>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="3"/>
-    </row>
-    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="2" t="s">
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="3"/>
-    </row>
-    <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="2" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="3"/>
-    </row>
-    <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="2" t="s">
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="3"/>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="2" t="s">
+    </row>
+    <row r="27" spans="1:2" ht="12.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="3"/>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-    </row>
-    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-    </row>
-    <row r="27" spans="1:2" ht="12.3" x14ac:dyDescent="0.4"/>
+    </row>
     <row r="28" spans="1:2" ht="12.3" x14ac:dyDescent="0.4"/>
     <row r="29" spans="1:2" ht="12.3" x14ac:dyDescent="0.4"/>
     <row r="30" spans="1:2" ht="12.3" x14ac:dyDescent="0.4"/>

</xml_diff>